<commit_message>
Merge глаза into Ozon pull request: close loss-making eye-signet line + storage cleanup
28 SKU / 94 units / забор 2820₽ one-time. Excludes profitable D493 earrings. Saves ~3092₽/mo storage plus stops loss-making глаза sales.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RB3ZzCvNjh49PbwKyrmhRr
</commit_message>
<xml_diff>
--- a/Таблицы/Заявка_вывоз_Ozon_хранение.xlsx
+++ b/Таблицы/Заявка_вывоз_Ozon_хранение.xlsx
@@ -57,17 +57,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00E4DFEC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,6 +123,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -490,29 +493,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Забор мёртвого товара с Озона — заявка на вывоз (чтобы не платить за хранение)</t>
+          <t>Забор товара с Озона — заявка на вывоз (хранение + закрытие линейки «глаза»)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Хранение всего ~6 850 ₽/мес. Мёртвый товар из этого = 3 091 ₽/мес. Забор разовый ~30 ₽/шт, окупается &lt;1 мес.</t>
+          <t>Забор ~30 ₽/шт. Причины: мёртвый товар жрёт хранение / глаза продаются в убыток — линейку закрываем.</t>
         </is>
       </c>
     </row>
@@ -529,550 +532,912 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Размер</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>Кол-во к вывозу</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Разовый забор ₽</t>
-        </is>
-      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Экономия ₽/мес</t>
+          <t>Забор ₽</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Окуп. мес</t>
+          <t>Экономия хранения ₽/мес</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Включить</t>
+          <t>Причина</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>D462-S</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Зеленый глаз»</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>хранение + глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
           <t>D519</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Сережки «Весенние тюльпаны»</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E6" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F6" s="6" t="n">
         <v>368</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>D535</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Сережки «Камилла»</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E7" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F7" s="6" t="n">
         <v>364</v>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>D529</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Кольцо «Ирис»</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E8" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F8" s="6" t="n">
         <v>318</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>D292</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Сережки «Винтаж»</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E9" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F9" s="6" t="n">
         <v>312</v>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>D528</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Кольцо «Ирис»</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E10" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F10" s="6" t="n">
         <v>265</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>D527</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Кольцо «Ирис»</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E11" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F11" s="6" t="n">
         <v>265</v>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>D236</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Сережки «Цикада»</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E12" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F12" s="6" t="n">
         <v>219</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>D518</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Сережки «Тропики»</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E13" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F13" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>D491</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Сережки «Катарина»</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E14" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F14" s="6" t="n">
         <v>165</v>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>D495</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Кольцо «Роза»</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E15" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F15" s="6" t="n">
         <v>138</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>MSH-013</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Сережки «Лучиана»</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E16" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F16" s="6" t="n">
         <v>110</v>
       </c>
-      <c r="F15" s="4" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>D507-S</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Сережки ассиметричные «Змеи»</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="E17" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="F17" s="6" t="n">
         <v>110</v>
       </c>
-      <c r="F16" s="4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>D520</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Сережки «Ночное небо»</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>101</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
+          <t>D520</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Сережки «Ночное небо»</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>101</v>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
           <t>D354</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Сережки «Ракушки»</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="E19" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="F19" s="6" t="n">
         <v>73</v>
       </c>
-      <c r="F18" s="6" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>На выбор</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>D462-S</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Кольцо-печатка «Зеленый глаз»</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n">
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>D494</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Кольцо «Роза»</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>D330</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Кольцо «Ника»</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="E21" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="E19" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>D494</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Кольцо «Роза»</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
+      <c r="F21" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>хранение</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>D503</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Глаз»</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>D505</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Глаз»</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>D256-S</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Взгляд»</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="E24" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="E20" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>D330</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Кольцо «Ника»</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F21" s="8" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>Пропустить</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>ИТОГО рекомендовано (Да):</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="n">
-        <v>69</v>
-      </c>
-      <c r="D23" s="10" t="n">
-        <v>2070</v>
-      </c>
-      <c r="E23" s="10" t="n">
-        <v>3011</v>
+      <c r="F24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Рекомендация: забрать 15 SKU (зелёные) — забор 2070 ₽ один раз, экономия 3011 ₽/мес.</t>
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>D466</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Карий глаз»</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F25" s="8" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>D354 Ракушки — «На выбор» (окуп. 4 мес, но продаётся на ВБ — можно забрать и переложить). D330 Ника — пропустить (8 ₽/мес).</t>
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>D449-S</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Голубой глаз»</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>D504</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Глаз»</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F27" s="8" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>D445-S</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Голубой глаз»</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F28" s="8" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>D007</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Голубой глаз»</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F29" s="8" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>D258-S</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Взгляд»</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F30" s="8" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>D375</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Взгляд»</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F31" s="8" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>D148</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо-печатка «Голубой глаз»</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F32" s="8" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>глаза (убыток)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>ИТОГО:</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n"/>
+      <c r="D34" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="E34" s="10" t="n">
+        <v>2820</v>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>3092</v>
+      </c>
+      <c r="G34" s="11" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Всего к вывозу: 94 шт, разовый забор 2820 ₽. Экономия хранения ~3092 ₽/мес.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>🟪 хранение+глаза · 🟧 только хранение · 🟩 только глаза (убыточная линейка). D493 «Сережки Глаза» НЕ включены — прибыльные (+580 ₽).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Отдельно: 7 печаток-глаз уже с 0 остатка на Озоне (D260, D448-S, D447-S, D259, D438-S, D439-S, D461-S) — вывозить нечего, просто не пополнять.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: exclude D539 (sells) from pull list — 41 SKU total
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RB3ZzCvNjh49PbwKyrmhRr
</commit_message>
<xml_diff>
--- a/Таблицы/Заявка_вывоз_Ozon_хранение.xlsx
+++ b/Таблицы/Заявка_вывоз_Ozon_хранение.xlsx
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Забираем всё: мёртвое (не продаётся) + все печатки/глаза. Забор ~30 ₽/шт, окупается меньше чем за месяц.</t>
+          <t>Забираем всё: мёртвое (не продаётся) + все печатки/глаза + 4 без данных. Забор ~30 ₽/шт.</t>
         </is>
       </c>
     </row>
@@ -751,26 +751,26 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>D539</t>
+          <t>D528</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Серьги повседневные изящные Муза и сосуд</t>
+          <t>Девушка с сережкой - Кольцо "Ирис"</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>256</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>не продаётся / нет данных</t>
+          <t>мёртвый (хранение)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -782,26 +782,26 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>D528</t>
+          <t>D467</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо "Ирис"</t>
+          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>256</v>
+        <v>239</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>мёртвый (хранение)</t>
+          <t>печатка/глаз</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -813,26 +813,26 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>D467</t>
+          <t>D236</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
+          <t>Серьги игривые летние Цикада</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>270</v>
+        <v>210</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>239</v>
+        <v>205</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>печатка/глаз</t>
+          <t>мёртвый (хранение)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -844,26 +844,26 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>D236</t>
+          <t>D304</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Серьги игривые летние Цикада</t>
+          <t>Серьги дизайнерские необычные повседневные "Слоны"</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>210</v>
+        <v>120</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>205</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>мёртвый (хранение)</t>
+          <t>нет данных о продажах</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>D304</t>
+          <t>D527</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Серьги дизайнерские необычные повседневные "Слоны"</t>
+          <t>Девушка с сережкой - Кольцо "Ирис"</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
@@ -894,7 +894,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>не продаётся / нет данных</t>
+          <t>мёртвый (хранение)</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -906,12 +906,12 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>D527</t>
+          <t>D518</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо "Ирис"</t>
+          <t>Серьги большие Тропики</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -937,22 +937,22 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>D518</t>
+          <t>MSH-013</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Серьги большие Тропики</t>
+          <t>Серьги стильные необычные висячие Лучиана</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
@@ -968,26 +968,26 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>MSH-013</t>
+          <t>D338</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Серьги стильные необычные висячие Лучиана</t>
+          <t>Кольцо-печатка крупное винтажное "Зеленый глаз"</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>мёртвый (хранение)</t>
+          <t>печатка/глаз</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -999,12 +999,12 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>D338</t>
+          <t>D468</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Зеленый глаз"</t>
+          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
@@ -1030,22 +1030,22 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>D468</t>
+          <t>D339</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
+          <t>Кольцо-печатка крупное винтажное "Голубой глаз"</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>D339</t>
+          <t>D341</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1092,7 +1092,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>D341</t>
+          <t>D436</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1123,12 +1123,12 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>D436</t>
+          <t>D453</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Голубой глаз"</t>
+          <t>Кольцо-печатка крупное винтажное "Зеленый глаз"</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
@@ -1154,12 +1154,12 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>D453</t>
+          <t>D495</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Зеленый глаз"</t>
+          <t>Девушка с сережкой - Кольцо "Роза"</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
@@ -1169,11 +1169,11 @@
         <v>180</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>160</v>
+        <v>133</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>печатка/глаз</t>
+          <t>мёртвый (хранение)</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1185,26 +1185,26 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>D495</t>
+          <t>D486-S</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо "Роза"</t>
+          <t>Кольцо-печатка серебристое "Карий глаз"</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>133</v>
+        <v>106</v>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>мёртвый (хранение)</t>
+          <t>печатка/глаз</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1216,26 +1216,26 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>D486-S</t>
+          <t>D491</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка серебристое "Карий глаз"</t>
+          <t>Серьги бижутерия необычные Катарина</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>печатка/глаз</t>
+          <t>мёртвый (хранение)</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1247,19 +1247,19 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>D491</t>
+          <t>D507-S</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Серьги бижутерия необычные Катарина</t>
+          <t>Серьги необычные вечерние Змеи</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>102</v>
@@ -1278,19 +1278,19 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>D507-S</t>
+          <t>D520</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Серьги необычные вечерние Змеи</t>
+          <t>Серьги винтажные необычные Ночное небо</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>102</v>
@@ -1309,26 +1309,26 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>D520</t>
+          <t>D437</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Серьги винтажные необычные Ночное небо</t>
+          <t>Кольцо-печатка крупное винтажное "Голубой глаз"</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>мёртвый (хранение)</t>
+          <t>печатка/глаз</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1340,26 +1340,26 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>D437</t>
+          <t>D162</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Голубой глаз"</t>
+          <t>Девушка с сережкой - Моносережка "Африка"</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>печатка/глаз</t>
+          <t>нет данных о продажах</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1371,12 +1371,12 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>D162</t>
+          <t>D333</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Моносережка "Африка"</t>
+          <t>Девушка с сережкой - Кольцо "Ключ"</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
@@ -1386,11 +1386,11 @@
         <v>120</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>не продаётся / нет данных</t>
+          <t>нет данных о продажах</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1402,7 +1402,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>D333</t>
+          <t>D334</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1411,17 +1411,17 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>53</v>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>не продаётся / нет данных</t>
+          <t>нет данных о продажах</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1433,26 +1433,26 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>D334</t>
+          <t>D463</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо "Ключ"</t>
+          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="E34" s="4" t="n">
         <v>53</v>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>не продаётся / нет данных</t>
+          <t>печатка/глаз</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1464,19 +1464,19 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>D463</t>
+          <t>D505</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
+          <t>Девушка с сережкой - Кольцо-печатка "Глаз"</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>53</v>
@@ -1495,22 +1495,22 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>D505</t>
+          <t>D382</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо-печатка "Глаз"</t>
+          <t>Девушка с сережкой - Кольцо-печатка "Северное возрождение"</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>D382</t>
+          <t>D386</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1557,12 +1557,12 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>D386</t>
+          <t>D434</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо-печатка "Северное возрождение"</t>
+          <t>Кольцо-печатка крупное винтажное "Голубой глаз"</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
@@ -1588,7 +1588,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>D434</t>
+          <t>D435</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1619,12 +1619,12 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>D435</t>
+          <t>D465</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Голубой глаз"</t>
+          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
@@ -1650,12 +1650,12 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>D465</t>
+          <t>D462-S</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка крупное винтажное "Карий глаз"</t>
+          <t>Кольцо-печатка серебристое "Зеленый глаз"</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
@@ -1681,12 +1681,12 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>D462-S</t>
+          <t>D487-S</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка серебристое "Зеленый глаз"</t>
+          <t>Кольцо-печатка серебристое "Карий глаз"</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
@@ -1712,12 +1712,12 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>D487-S</t>
+          <t>D494</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Кольцо-печатка серебристое "Карий глаз"</t>
+          <t>Девушка с сережкой - Кольцо "Роза"</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>печатка/глаз</t>
+          <t>мёртвый (хранение)</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -1743,12 +1743,12 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>D494</t>
+          <t>D503</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо "Роза"</t>
+          <t>Девушка с сережкой - Кольцо-печатка "Глаз"</t>
         </is>
       </c>
       <c r="C44" s="4" t="n">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>мёртвый (хранение)</t>
+          <t>печатка/глаз</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -1774,26 +1774,26 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>D503</t>
+          <t>D330</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Девушка с сережкой - Кольцо-печатка "Глаз"</t>
+          <t>Девушка с сережкой - Кольцо "Ника"</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>печатка/глаз</t>
+          <t>мёртвый (хранение)</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -1802,57 +1802,33 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>D330</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Девушка с сережкой - Кольцо "Ника"</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D46" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>мёртвый (хранение)</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>Запланировано</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="6" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>ИТОГО:</t>
         </is>
       </c>
-      <c r="C48" s="6" t="n">
-        <v>186</v>
-      </c>
-      <c r="D48" s="6" t="n">
-        <v>5580</v>
-      </c>
-      <c r="E48" s="6" t="n">
-        <v>6132</v>
+      <c r="C47" s="6" t="n">
+        <v>181</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>5430</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>5876</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Всего к вывозу: 41 SKU, 181 шт. Разовый забор 5,430 ₽. Экономия хранения 5,876 ₽/мес — окупается ~за 3 недели.</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Всего к вывозу: 42 SKU, 186 шт. Разовый забор 5,580 ₽. Экономия хранения 6,132 ₽/мес — окупается ~за 3 недели.</t>
+          <t>Не забираем: Серьги повседневные изящные Муза и сосуд — продаётся, уйдёт сам.</t>
         </is>
       </c>
     </row>

</xml_diff>